<commit_message>
re-run test sebelum demo besok pagi
</commit_message>
<xml_diff>
--- a/sd_kediri.xlsx
+++ b/sd_kediri.xlsx
@@ -716,7 +716,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>SDN Karangtalun 1</t>
+          <t>SDN KARANGTALUN 1</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1261,7 +1261,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Jl. Merak 83</t>
+          <t>Jl. Merak</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1661,7 +1661,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Margourip</t>
+          <t>Dusun Margourip</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -2501,7 +2501,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Dsn Bogor Pradah</t>
+          <t>Jl. Raya Besowo No. 158, Dsn Bogorpradah</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -4581,7 +4581,7 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>Jalan Branjangan</t>
+          <t>Jalan Gelatik No. 120</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
@@ -8616,7 +8616,7 @@
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>SDN Gabru</t>
+          <t>SDN GABRU</t>
         </is>
       </c>
       <c r="C410" t="inlineStr">
@@ -10901,7 +10901,7 @@
       </c>
       <c r="C524" t="inlineStr">
         <is>
-          <t>Dsn. Borolor</t>
+          <t>Jl. Raya Kunjang - Gudo Dusun Borolor</t>
         </is>
       </c>
       <c r="D524" t="inlineStr">
@@ -16201,7 +16201,7 @@
       </c>
       <c r="C789" t="inlineStr">
         <is>
-          <t>Jl. Letjen Suprapto No. 3</t>
+          <t>Jl. Letjend Suprapto No. 3</t>
         </is>
       </c>
       <c r="D789" t="inlineStr">

</xml_diff>